<commit_message>
Calendario: Se agendó ARTE (11:00 - 13:00) para 26/05/2026
</commit_message>
<xml_diff>
--- a/calendario.xlsx
+++ b/calendario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,11 @@
           <t>HORAS</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>HORARIO</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -457,6 +462,7 @@
       <c r="D2" t="n">
         <v>1</v>
       </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -477,6 +483,7 @@
       <c r="D3" t="n">
         <v>1</v>
       </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -497,6 +504,7 @@
       <c r="D4" t="n">
         <v>1</v>
       </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -517,6 +525,7 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -537,6 +546,7 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -557,6 +567,7 @@
       <c r="D7" t="n">
         <v>1</v>
       </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -576,6 +587,232 @@
       </c>
       <c r="D8" t="n">
         <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>11:00 - 13:00</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calendario: Se agendó ARTE (10:30 - 12:30) para 27/05/2026
</commit_message>
<xml_diff>
--- a/calendario.xlsx
+++ b/calendario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1040,6 +1040,306 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Calendario: Se agendó TALLER "SÍ PUEDO" (10:00 - 12:00) para 23/05/2026
</commit_message>
<xml_diff>
--- a/calendario.xlsx
+++ b/calendario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1340,6 +1340,231 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>TALLER "SÍ PUEDO"</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>10:00 - 12:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Calendario: Se agendó TEATRO (10:30 - 12:30) para 23/05/2026
</commit_message>
<xml_diff>
--- a/calendario.xlsx
+++ b/calendario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1565,6 +1565,81 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TEATRO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TEATRO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>TEATRO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Calendario: Se agendó GRUPO DE CRECIMIENTO (10:30 - 11:30) para 23/05/2026
</commit_message>
<xml_diff>
--- a/calendario.xlsx
+++ b/calendario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1640,6 +1640,81 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>10:30 - 11:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>10:30 - 11:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>GRUPO DE CRECIMIENTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>10:30 - 11:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Calendario: Modificación bloque ARTE
</commit_message>
<xml_diff>
--- a/calendario.xlsx
+++ b/calendario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1043,7 +1043,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1061,24 +1061,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1086,24 +1086,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
+          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1111,24 +1111,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>FERNANDO ÁVILA BERLANGA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1136,24 +1136,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1161,24 +1161,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GUADALUPE LÓPEZ TOVAR</t>
+          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1186,24 +1186,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1211,24 +1211,24 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1236,24 +1236,24 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TALLER "SÍ PUEDO"</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1261,24 +1261,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>10:30 - 12:30</t>
+          <t>10:00 - 12:00</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TEATRO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1293,17 +1293,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TEATRO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1318,17 +1318,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
+          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ARTE</t>
+          <t>TEATRO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1348,20 +1348,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
+          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>GRUPO DE CRECIMIENTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 11:30</t>
         </is>
       </c>
     </row>
@@ -1373,20 +1373,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>FLORINDA ESTEVANÉ PIZARRO</t>
+          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>GRUPO DE CRECIMIENTO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 11:30</t>
         </is>
       </c>
     </row>
@@ -1398,37 +1398,37 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>JESÚS ALEJANDRO SIFUENTES ESPINO</t>
+          <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>GRUPO DE CRECIMIENTO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 11:30</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
+          <t>ANA DE LOS ÁNGELES TORRES REVELES</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1436,24 +1436,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
+          <t>CARLOS ALBERTO DE LA TORRE SANTELLANO</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1461,24 +1461,24 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>JUAN SILVERIO LÓPEZ DE LA ROSA</t>
+          <t>CRISTABEL DE LA CRUZ MALDONADO</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1486,24 +1486,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>KARLA LISSETTE PEDROZA GONZÁLEZ</t>
+          <t>FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1511,24 +1511,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
+          <t>FLORINDA ESTEVANÉ PIZARRO</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1536,24 +1536,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>GUADALUPE LÓPEZ TOVAR</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>TALLER "SÍ PUEDO"</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1561,24 +1561,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>10:00 - 12:00</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>JUAN RAFAEL YAÑEZ SERNA</t>
+          <t>JOSE REYNALDO ALCORTA BENAVIDES</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1593,17 +1593,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+          <t>JUAN JOSÉ OCHOA GONZÁLEZ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1618,17 +1618,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MARÍA GUADALUPE DE LA CONCEPCIÓN TORRES LIRA</t>
+          <t>JUAN RAFAEL YAÑEZ SERNA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TEATRO</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1643,75 +1643,125 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MARÍA DE LOS ÁNGELES ORDUÑA RODRÍGUEZ</t>
+          <t>LUIS FERNANDO ÁVILA BERLANGA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>GRUPO DE CRECIMIENTO</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>10:30 - 11:30</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PEDRO ANTONIO DE LA CERDA TREVIÑO</t>
+          <t>LUIS JAVIER GARCÍA MARTÍNEZ</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>GRUPO DE CRECIMIENTO</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>10:30 - 11:30</t>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>MA. ELIZABETH GONZÁLEZ HIDROGO</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>TERESITA DEL NIÑO JESÚS RODRÍGUEZ SALAZAR</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>TOMASITA MARÍA ENRIQUETA RIVERA DEL BOSQUE</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>GRUPO DE CRECIMIENTO</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>10:30 - 11:30</t>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ARTE</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>10:30 - 12:30</t>
         </is>
       </c>
     </row>

</xml_diff>